<commit_message>
Add monthly package and secondment status
</commit_message>
<xml_diff>
--- a/projects/PetroUrdaneta-FDP9/compensation/source_annual_compensation_table.xlsx
+++ b/projects/PetroUrdaneta-FDP9/compensation/source_annual_compensation_table.xlsx
@@ -9,11 +9,15 @@
   </bookViews>
   <sheets>
     <sheet name="Annual Package" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Monthly Package" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Annual Package'!$A$1:$J$11</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Annual Package'!$A$1:$K$11</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Annual Package'!$1:$1</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Annual Package'!$A$1:$J$10</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Annual Package'!$A$1:$K$10</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Monthly Package'!$A$1:$K$11</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">'Monthly Package'!$1:$1</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Monthly Package'!$A$1:$K$10</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -67,8 +71,51 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Monthly values are calculated as annual component divided by 12.</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>37</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>2</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>-121</xdr:colOff>
+                <xdr:row>1</xdr:row>
+                <xdr:rowOff>25</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="40">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -100,12 +147,18 @@
     <t xml:space="preserve">TOTAL Annual Package</t>
   </si>
   <si>
+    <t xml:space="preserve">Secondment Status</t>
+  </si>
+  <si>
     <t xml:space="preserve">COO / PU General Manager</t>
   </si>
   <si>
     <t xml:space="preserve">Martin del Castillo</t>
   </si>
   <si>
+    <t xml:space="preserve">Not Secondee</t>
+  </si>
+  <si>
     <t xml:space="preserve">EPCM &amp; Engineering Manager</t>
   </si>
   <si>
@@ -118,6 +171,9 @@
     <t xml:space="preserve">Alexander Stulme</t>
   </si>
   <si>
+    <t xml:space="preserve">Secondee</t>
+  </si>
+  <si>
     <t xml:space="preserve">Operations &amp; Maintenance Manager</t>
   </si>
   <si>
@@ -155,15 +211,40 @@
   </si>
   <si>
     <t xml:space="preserve">TOTAL ANNUAL COST (9 positions)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base Salary (Monthly)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Housing (Monthly)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medical Insurance (Monthly)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home Leave (Monthly)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company Vehicle (Monthly)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tax &amp; Social (Monthly)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL Monthly Package</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL MONTHLY COST (9 positions)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0;[RED]&quot;($&quot;#,##0\);\-"/>
+    <numFmt numFmtId="166" formatCode="\$#,##0.00;[RED]&quot;($&quot;#,##0.00\);\-"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -304,7 +385,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -329,6 +410,10 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -345,6 +430,10 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -354,6 +443,26 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -474,10 +583,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AnnualCompensationTable" displayName="AnnualCompensationTable" ref="A1:J10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:J10"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AnnualCompensationTable" displayName="AnnualCompensationTable" ref="A1:K10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:K10"/>
+  <tableColumns count="11">
     <tableColumn id="1" name="#"/>
     <tableColumn id="2" name="Position"/>
     <tableColumn id="3" name="Person"/>
@@ -488,6 +601,26 @@
     <tableColumn id="8" name="Company Vehicle"/>
     <tableColumn id="9" name="Tax &amp; Social"/>
     <tableColumn id="10" name="TOTAL Annual Package"/>
+    <tableColumn id="11" name="Secondment Status"/>
+  </tableColumns>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="MonthlyCompensationTable" displayName="MonthlyCompensationTable" ref="A1:K10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:K10"/>
+  <tableColumns count="11">
+    <tableColumn id="1" name="#"/>
+    <tableColumn id="2" name="Position"/>
+    <tableColumn id="3" name="Person"/>
+    <tableColumn id="4" name="Base Salary (Monthly)"/>
+    <tableColumn id="5" name="Housing (Monthly)"/>
+    <tableColumn id="6" name="Medical Insurance (Monthly)"/>
+    <tableColumn id="7" name="Home Leave (Monthly)"/>
+    <tableColumn id="8" name="Company Vehicle (Monthly)"/>
+    <tableColumn id="9" name="Tax &amp; Social (Monthly)"/>
+    <tableColumn id="10" name="TOTAL Monthly Package"/>
+    <tableColumn id="11" name="Secondment Status"/>
   </tableColumns>
 </table>
 </file>
@@ -672,7 +805,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -684,6 +817,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -717,16 +851,19 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" s="4" t="n">
         <v>360000</v>
@@ -750,38 +887,44 @@
         <f aca="false">SUM(D2:I2)</f>
         <v>524000</v>
       </c>
+      <c r="K2" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="n">
+      <c r="A3" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" s="8" t="n">
+      <c r="B3" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="9" t="n">
         <v>216000</v>
       </c>
-      <c r="E3" s="8" t="n">
+      <c r="E3" s="9" t="n">
         <v>24000</v>
       </c>
-      <c r="F3" s="8" t="n">
+      <c r="F3" s="9" t="n">
         <v>12000</v>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G3" s="9" t="n">
         <v>12000</v>
       </c>
-      <c r="H3" s="8" t="n">
+      <c r="H3" s="9" t="n">
         <v>18000</v>
       </c>
-      <c r="I3" s="8" t="n">
+      <c r="I3" s="9" t="n">
         <v>43200</v>
       </c>
-      <c r="J3" s="9" t="n">
+      <c r="J3" s="10" t="n">
         <f aca="false">SUM(D3:I3)</f>
         <v>325200</v>
+      </c>
+      <c r="K3" s="11" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -789,10 +932,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>180000</v>
@@ -816,38 +959,44 @@
         <f aca="false">SUM(D4:I4)</f>
         <v>282000</v>
       </c>
+      <c r="K4" s="6" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="8" t="n">
+      <c r="B5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="9" t="n">
         <v>216000</v>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="9" t="n">
         <v>24000</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F5" s="9" t="n">
         <v>12000</v>
       </c>
-      <c r="G5" s="8" t="n">
+      <c r="G5" s="9" t="n">
         <v>12000</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="H5" s="9" t="n">
         <v>18000</v>
       </c>
-      <c r="I5" s="8" t="n">
+      <c r="I5" s="9" t="n">
         <v>43200</v>
       </c>
-      <c r="J5" s="9" t="n">
+      <c r="J5" s="10" t="n">
         <f aca="false">SUM(D5:I5)</f>
         <v>325200</v>
+      </c>
+      <c r="K5" s="11" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -855,10 +1004,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>180000</v>
@@ -882,38 +1031,44 @@
         <f aca="false">SUM(D6:I6)</f>
         <v>282000</v>
       </c>
+      <c r="K6" s="6" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="8" t="n">
+      <c r="B7" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="9" t="n">
         <v>120000</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="9" t="n">
         <v>18000</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F7" s="9" t="n">
         <v>12000</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="G7" s="9" t="n">
         <v>12000</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="9" t="n">
         <v>12000</v>
       </c>
-      <c r="I7" s="8" t="n">
+      <c r="I7" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="J7" s="9" t="n">
+      <c r="J7" s="10" t="n">
         <f aca="false">SUM(D7:I7)</f>
         <v>194000</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -921,10 +1076,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>180000</v>
@@ -948,38 +1103,44 @@
         <f aca="false">SUM(D8:I8)</f>
         <v>282000</v>
       </c>
+      <c r="K8" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D9" s="8" t="n">
+      <c r="B9" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="9" t="n">
         <v>48000</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="9" t="n">
         <v>12000</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F9" s="9" t="n">
         <v>8000</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="H9" s="9" t="n">
         <v>7200</v>
       </c>
-      <c r="I9" s="8" t="n">
+      <c r="I9" s="9" t="n">
         <v>12000</v>
       </c>
-      <c r="J9" s="9" t="n">
+      <c r="J9" s="10" t="n">
         <f aca="false">SUM(D9:I9)</f>
         <v>87200</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -987,10 +1148,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>48000</v>
@@ -1014,26 +1175,30 @@
         <f aca="false">SUM(D10:I10)</f>
         <v>95200</v>
       </c>
+      <c r="K10" s="6" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="12" t="n">
+      <c r="A11" s="12"/>
+      <c r="B11" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="14" t="n">
         <f aca="false">SUM(J2:J10)</f>
         <v>2396800</v>
       </c>
+      <c r="K11" s="12"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J10"/>
+  <autoFilter ref="A1:K10"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.5"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1047,4 +1212,508 @@
     <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="n">
+        <f aca="false">'Annual Package'!A2</f>
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="str">
+        <f aca="false">'Annual Package'!B2</f>
+        <v>COO / PU General Manager</v>
+      </c>
+      <c r="C2" s="3" t="str">
+        <f aca="false">'Annual Package'!C2</f>
+        <v>Martin del Castillo</v>
+      </c>
+      <c r="D2" s="15" t="n">
+        <f aca="false">'Annual Package'!D2/12</f>
+        <v>30000</v>
+      </c>
+      <c r="E2" s="15" t="n">
+        <f aca="false">'Annual Package'!E2/12</f>
+        <v>3000</v>
+      </c>
+      <c r="F2" s="15" t="n">
+        <f aca="false">'Annual Package'!F2/12</f>
+        <v>1000</v>
+      </c>
+      <c r="G2" s="15" t="n">
+        <f aca="false">'Annual Package'!G2/12</f>
+        <v>1666.66666666667</v>
+      </c>
+      <c r="H2" s="15" t="n">
+        <f aca="false">'Annual Package'!H2/12</f>
+        <v>2000</v>
+      </c>
+      <c r="I2" s="15" t="n">
+        <f aca="false">'Annual Package'!I2/12</f>
+        <v>6000</v>
+      </c>
+      <c r="J2" s="16" t="n">
+        <f aca="false">SUM(D2:I2)</f>
+        <v>43666.6666666667</v>
+      </c>
+      <c r="K2" s="6" t="str">
+        <f aca="false">'Annual Package'!K2</f>
+        <v>Not Secondee</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="n">
+        <f aca="false">'Annual Package'!A3</f>
+        <v>2</v>
+      </c>
+      <c r="B3" s="8" t="str">
+        <f aca="false">'Annual Package'!B3</f>
+        <v>EPCM &amp; Engineering Manager</v>
+      </c>
+      <c r="C3" s="8" t="str">
+        <f aca="false">'Annual Package'!C3</f>
+        <v>Juan Conde</v>
+      </c>
+      <c r="D3" s="17" t="n">
+        <f aca="false">'Annual Package'!D3/12</f>
+        <v>18000</v>
+      </c>
+      <c r="E3" s="17" t="n">
+        <f aca="false">'Annual Package'!E3/12</f>
+        <v>2000</v>
+      </c>
+      <c r="F3" s="17" t="n">
+        <f aca="false">'Annual Package'!F3/12</f>
+        <v>1000</v>
+      </c>
+      <c r="G3" s="17" t="n">
+        <f aca="false">'Annual Package'!G3/12</f>
+        <v>1000</v>
+      </c>
+      <c r="H3" s="17" t="n">
+        <f aca="false">'Annual Package'!H3/12</f>
+        <v>1500</v>
+      </c>
+      <c r="I3" s="17" t="n">
+        <f aca="false">'Annual Package'!I3/12</f>
+        <v>3600</v>
+      </c>
+      <c r="J3" s="18" t="n">
+        <f aca="false">SUM(D3:I3)</f>
+        <v>27100</v>
+      </c>
+      <c r="K3" s="11" t="str">
+        <f aca="false">'Annual Package'!K3</f>
+        <v>Not Secondee</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="n">
+        <f aca="false">'Annual Package'!A4</f>
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="str">
+        <f aca="false">'Annual Package'!B4</f>
+        <v>Drilling &amp; Well Services Manager</v>
+      </c>
+      <c r="C4" s="3" t="str">
+        <f aca="false">'Annual Package'!C4</f>
+        <v>Alexander Stulme</v>
+      </c>
+      <c r="D4" s="15" t="n">
+        <f aca="false">'Annual Package'!D4/12</f>
+        <v>15000</v>
+      </c>
+      <c r="E4" s="15" t="n">
+        <f aca="false">'Annual Package'!E4/12</f>
+        <v>2000</v>
+      </c>
+      <c r="F4" s="15" t="n">
+        <f aca="false">'Annual Package'!F4/12</f>
+        <v>1000</v>
+      </c>
+      <c r="G4" s="15" t="n">
+        <f aca="false">'Annual Package'!G4/12</f>
+        <v>1000</v>
+      </c>
+      <c r="H4" s="15" t="n">
+        <f aca="false">'Annual Package'!H4/12</f>
+        <v>1500</v>
+      </c>
+      <c r="I4" s="15" t="n">
+        <f aca="false">'Annual Package'!I4/12</f>
+        <v>3000</v>
+      </c>
+      <c r="J4" s="16" t="n">
+        <f aca="false">SUM(D4:I4)</f>
+        <v>23500</v>
+      </c>
+      <c r="K4" s="6" t="str">
+        <f aca="false">'Annual Package'!K4</f>
+        <v>Secondee</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="n">
+        <f aca="false">'Annual Package'!A5</f>
+        <v>4</v>
+      </c>
+      <c r="B5" s="8" t="str">
+        <f aca="false">'Annual Package'!B5</f>
+        <v>Operations &amp; Maintenance Manager</v>
+      </c>
+      <c r="C5" s="8" t="str">
+        <f aca="false">'Annual Package'!C5</f>
+        <v>Félix Valderrama</v>
+      </c>
+      <c r="D5" s="17" t="n">
+        <f aca="false">'Annual Package'!D5/12</f>
+        <v>18000</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <f aca="false">'Annual Package'!E5/12</f>
+        <v>2000</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <f aca="false">'Annual Package'!F5/12</f>
+        <v>1000</v>
+      </c>
+      <c r="G5" s="17" t="n">
+        <f aca="false">'Annual Package'!G5/12</f>
+        <v>1000</v>
+      </c>
+      <c r="H5" s="17" t="n">
+        <f aca="false">'Annual Package'!H5/12</f>
+        <v>1500</v>
+      </c>
+      <c r="I5" s="17" t="n">
+        <f aca="false">'Annual Package'!I5/12</f>
+        <v>3600</v>
+      </c>
+      <c r="J5" s="18" t="n">
+        <f aca="false">SUM(D5:I5)</f>
+        <v>27100</v>
+      </c>
+      <c r="K5" s="11" t="str">
+        <f aca="false">'Annual Package'!K5</f>
+        <v>Not Secondee</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="n">
+        <f aca="false">'Annual Package'!A6</f>
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="str">
+        <f aca="false">'Annual Package'!B6</f>
+        <v>Technical Manager (Geosciences)</v>
+      </c>
+      <c r="C6" s="3" t="str">
+        <f aca="false">'Annual Package'!C6</f>
+        <v>Alan McKeon</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <f aca="false">'Annual Package'!D6/12</f>
+        <v>15000</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <f aca="false">'Annual Package'!E6/12</f>
+        <v>2000</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <f aca="false">'Annual Package'!F6/12</f>
+        <v>1000</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <f aca="false">'Annual Package'!G6/12</f>
+        <v>1000</v>
+      </c>
+      <c r="H6" s="15" t="n">
+        <f aca="false">'Annual Package'!H6/12</f>
+        <v>1500</v>
+      </c>
+      <c r="I6" s="15" t="n">
+        <f aca="false">'Annual Package'!I6/12</f>
+        <v>3000</v>
+      </c>
+      <c r="J6" s="16" t="n">
+        <f aca="false">SUM(D6:I6)</f>
+        <v>23500</v>
+      </c>
+      <c r="K6" s="6" t="str">
+        <f aca="false">'Annual Package'!K6</f>
+        <v>Secondee</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="n">
+        <f aca="false">'Annual Package'!A7</f>
+        <v>6</v>
+      </c>
+      <c r="B7" s="8" t="str">
+        <f aca="false">'Annual Package'!B7</f>
+        <v>Reservoir Engineer</v>
+      </c>
+      <c r="C7" s="8" t="str">
+        <f aca="false">'Annual Package'!C7</f>
+        <v>JJI</v>
+      </c>
+      <c r="D7" s="17" t="n">
+        <f aca="false">'Annual Package'!D7/12</f>
+        <v>10000</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <f aca="false">'Annual Package'!E7/12</f>
+        <v>1500</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <f aca="false">'Annual Package'!F7/12</f>
+        <v>1000</v>
+      </c>
+      <c r="G7" s="17" t="n">
+        <f aca="false">'Annual Package'!G7/12</f>
+        <v>1000</v>
+      </c>
+      <c r="H7" s="17" t="n">
+        <f aca="false">'Annual Package'!H7/12</f>
+        <v>1000</v>
+      </c>
+      <c r="I7" s="17" t="n">
+        <f aca="false">'Annual Package'!I7/12</f>
+        <v>1666.66666666667</v>
+      </c>
+      <c r="J7" s="18" t="n">
+        <f aca="false">SUM(D7:I7)</f>
+        <v>16166.6666666667</v>
+      </c>
+      <c r="K7" s="11" t="str">
+        <f aca="false">'Annual Package'!K7</f>
+        <v>Not Secondee</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="n">
+        <f aca="false">'Annual Package'!A8</f>
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="str">
+        <f aca="false">'Annual Package'!B8</f>
+        <v>Rig Company Man</v>
+      </c>
+      <c r="C8" s="3" t="str">
+        <f aca="false">'Annual Package'!C8</f>
+        <v>Marcelo Dantas</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <f aca="false">'Annual Package'!D8/12</f>
+        <v>15000</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <f aca="false">'Annual Package'!E8/12</f>
+        <v>2000</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <f aca="false">'Annual Package'!F8/12</f>
+        <v>1000</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <f aca="false">'Annual Package'!G8/12</f>
+        <v>1000</v>
+      </c>
+      <c r="H8" s="15" t="n">
+        <f aca="false">'Annual Package'!H8/12</f>
+        <v>1500</v>
+      </c>
+      <c r="I8" s="15" t="n">
+        <f aca="false">'Annual Package'!I8/12</f>
+        <v>3000</v>
+      </c>
+      <c r="J8" s="16" t="n">
+        <f aca="false">SUM(D8:I8)</f>
+        <v>23500</v>
+      </c>
+      <c r="K8" s="6" t="str">
+        <f aca="false">'Annual Package'!K8</f>
+        <v>Not Secondee</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="n">
+        <f aca="false">'Annual Package'!A9</f>
+        <v>8</v>
+      </c>
+      <c r="B9" s="8" t="str">
+        <f aca="false">'Annual Package'!B9</f>
+        <v>Planning &amp; PMO</v>
+      </c>
+      <c r="C9" s="8" t="str">
+        <f aca="false">'Annual Package'!C9</f>
+        <v>Jose Miguel</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <f aca="false">'Annual Package'!D9/12</f>
+        <v>4000</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <f aca="false">'Annual Package'!E9/12</f>
+        <v>1000</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <f aca="false">'Annual Package'!F9/12</f>
+        <v>666.666666666667</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <f aca="false">'Annual Package'!G9/12</f>
+        <v>0</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <f aca="false">'Annual Package'!H9/12</f>
+        <v>600</v>
+      </c>
+      <c r="I9" s="17" t="n">
+        <f aca="false">'Annual Package'!I9/12</f>
+        <v>1000</v>
+      </c>
+      <c r="J9" s="18" t="n">
+        <f aca="false">SUM(D9:I9)</f>
+        <v>7266.66666666667</v>
+      </c>
+      <c r="K9" s="11" t="str">
+        <f aca="false">'Annual Package'!K9</f>
+        <v>Not Secondee</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="n">
+        <f aca="false">'Annual Package'!A10</f>
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="str">
+        <f aca="false">'Annual Package'!B10</f>
+        <v>Operations Support</v>
+      </c>
+      <c r="C10" s="3" t="str">
+        <f aca="false">'Annual Package'!C10</f>
+        <v>Leticia Almeida</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <f aca="false">'Annual Package'!D10/12</f>
+        <v>4000</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <f aca="false">'Annual Package'!E10/12</f>
+        <v>1000</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <f aca="false">'Annual Package'!F10/12</f>
+        <v>666.666666666667</v>
+      </c>
+      <c r="G10" s="15" t="n">
+        <f aca="false">'Annual Package'!G10/12</f>
+        <v>1000</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <f aca="false">'Annual Package'!H10/12</f>
+        <v>600</v>
+      </c>
+      <c r="I10" s="15" t="n">
+        <f aca="false">'Annual Package'!I10/12</f>
+        <v>666.666666666667</v>
+      </c>
+      <c r="J10" s="16" t="n">
+        <f aca="false">SUM(D10:I10)</f>
+        <v>7933.33333333333</v>
+      </c>
+      <c r="K10" s="6" t="str">
+        <f aca="false">'Annual Package'!K10</f>
+        <v>Not Secondee</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12"/>
+      <c r="B11" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="19" t="n">
+        <f aca="false">SUM(J2:J10)</f>
+        <v>199733.333333333</v>
+      </c>
+      <c r="K11" s="12"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K10"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.5"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 &amp;K666666Monthly Package | Page &amp;P of &amp;N</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
+  <tableParts>
+    <tablePart r:id="rId4"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>